<commit_message>
DOC:Avance con especificación de CU. Casi completo
</commit_message>
<xml_diff>
--- a/A-Documentacion/A-Inicio/Iteracion1-31_8-al-20_9/eGraduados_Inicio_Iteracion1_PlanificacionTemporal.xlsx
+++ b/A-Documentacion/A-Inicio/Iteracion1-31_8-al-20_9/eGraduados_Inicio_Iteracion1_PlanificacionTemporal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\eGraduados\A-Documentacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\eGraduados\A-Documentacion\A-Inicio\Iteracion1-31_8-al-20_9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB2AD390-36B7-4308-A8B4-D9AB38D4CD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F099C7-2E7F-4DEC-891C-4BFFC80B1CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{C157A7F2-5B1B-4E06-B43B-1F6A14E9BE8B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Identificador</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>Identificar y descrbir modulos del sistema</t>
+  </si>
+  <si>
+    <t>Especificar Casos de Uso del sistema</t>
   </si>
 </sst>
 </file>
@@ -118,7 +121,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -128,6 +131,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -159,15 +180,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -502,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAB9D6C9-D4CB-4415-A5A6-1ABCE4095E7E}">
-  <dimension ref="C3:J13"/>
+  <dimension ref="C3:J14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -516,40 +542,40 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
     </row>
     <row r="4" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="4" t="s">
         <v>8</v>
       </c>
     </row>
@@ -571,7 +597,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
+      <c r="J5" s="8"/>
     </row>
     <row r="6" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C6" s="1">
@@ -591,7 +617,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
+      <c r="J6" s="9"/>
     </row>
     <row r="7" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C7" s="1">
@@ -613,7 +639,7 @@
       <c r="I7" s="1">
         <v>2</v>
       </c>
-      <c r="J7" s="1"/>
+      <c r="J7" s="9"/>
     </row>
     <row r="8" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C8" s="1">
@@ -635,58 +661,58 @@
       <c r="I8" s="1">
         <v>1</v>
       </c>
-      <c r="J8" s="1"/>
+      <c r="J8" s="9"/>
     </row>
     <row r="9" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C9" s="1">
+      <c r="C9" s="6">
         <v>5</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>18</v>
+      <c r="D9" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="E9" s="2">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="F9" s="2">
-        <v>46282</v>
-      </c>
-      <c r="G9" s="1">
+        <v>46283</v>
+      </c>
+      <c r="G9" s="6">
         <v>1</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1">
         <v>4</v>
       </c>
-      <c r="J9" s="1"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C10" s="1">
         <v>6</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>15</v>
+      <c r="D10" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="E10" s="2">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="F10" s="2">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="G10" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="1"/>
-      <c r="I10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J10" s="1"/>
+      <c r="I10" s="1">
+        <v>4</v>
+      </c>
+      <c r="J10" s="9"/>
     </row>
     <row r="11" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C11" s="1">
         <v>7</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>12</v>
+      <c r="D11" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="E11" s="2">
         <v>46283</v>
@@ -695,18 +721,20 @@
         <v>46283</v>
       </c>
       <c r="G11" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="I11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" s="9"/>
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C12" s="1">
         <v>8</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E12" s="2">
         <v>46283</v>
@@ -715,35 +743,55 @@
         <v>46283</v>
       </c>
       <c r="G12" s="1">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="H12" s="1"/>
-      <c r="I12" s="1">
-        <v>3</v>
-      </c>
-      <c r="J12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="10"/>
     </row>
     <row r="13" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C13" s="1">
         <v>9</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>17</v>
+      <c r="D13" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="E13" s="2">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="F13" s="2">
-        <v>46285</v>
+        <v>46283</v>
       </c>
       <c r="G13" s="1">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1">
+        <v>3</v>
+      </c>
+      <c r="J13" s="9"/>
+    </row>
+    <row r="14" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="6">
+        <v>10</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="2">
+        <v>46284</v>
+      </c>
+      <c r="F14" s="2">
+        <v>46285</v>
+      </c>
+      <c r="G14" s="1">
+        <v>2</v>
+      </c>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1">
         <v>6</v>
       </c>
-      <c r="J13" s="1"/>
+      <c r="J14" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
DOC: Actualización de planificación temporal
</commit_message>
<xml_diff>
--- a/A-Documentacion/A-Inicio/Iteracion1-31_8-al-20_9/eGraduados_Inicio_Iteracion1_PlanificacionTemporal.xlsx
+++ b/A-Documentacion/A-Inicio/Iteracion1-31_8-al-20_9/eGraduados_Inicio_Iteracion1_PlanificacionTemporal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\eGraduados\A-Documentacion\A-Inicio\Iteracion1-31_8-al-20_9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F099C7-2E7F-4DEC-891C-4BFFC80B1CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2293724D-AE2C-4654-99A5-8BEDFDF513CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{C157A7F2-5B1B-4E06-B43B-1F6A14E9BE8B}"/>
   </bookViews>
@@ -180,20 +180,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -542,16 +540,16 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
@@ -597,7 +595,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="8"/>
+      <c r="J5" s="5"/>
     </row>
     <row r="6" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C6" s="1">
@@ -617,7 +615,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="9"/>
+      <c r="J6" s="6"/>
     </row>
     <row r="7" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C7" s="1">
@@ -639,7 +637,7 @@
       <c r="I7" s="1">
         <v>2</v>
       </c>
-      <c r="J7" s="9"/>
+      <c r="J7" s="6"/>
     </row>
     <row r="8" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C8" s="1">
@@ -661,13 +659,13 @@
       <c r="I8" s="1">
         <v>1</v>
       </c>
-      <c r="J8" s="9"/>
+      <c r="J8" s="6"/>
     </row>
     <row r="9" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C9" s="6">
+      <c r="C9" s="1">
         <v>5</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="2">
@@ -676,14 +674,14 @@
       <c r="F9" s="2">
         <v>46283</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="1">
         <v>1</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1">
         <v>4</v>
       </c>
-      <c r="J9" s="9"/>
+      <c r="J9" s="5"/>
     </row>
     <row r="10" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C10" s="1">
@@ -705,7 +703,7 @@
       <c r="I10" s="1">
         <v>4</v>
       </c>
-      <c r="J10" s="9"/>
+      <c r="J10" s="5"/>
     </row>
     <row r="11" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C11" s="1">
@@ -727,7 +725,7 @@
       <c r="I11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="9"/>
+      <c r="J11" s="7"/>
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C12" s="1">
@@ -747,7 +745,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="10"/>
+      <c r="J12" s="7"/>
     </row>
     <row r="13" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C13" s="1">
@@ -769,10 +767,10 @@
       <c r="I13" s="1">
         <v>3</v>
       </c>
-      <c r="J13" s="9"/>
+      <c r="J13" s="6"/>
     </row>
     <row r="14" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C14" s="6">
+      <c r="C14" s="1">
         <v>10</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -791,7 +789,7 @@
       <c r="I14" s="1">
         <v>6</v>
       </c>
-      <c r="J14" s="1"/>
+      <c r="J14" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
DOC: Cierre de la iteración
</commit_message>
<xml_diff>
--- a/A-Documentacion/A-Inicio/Iteracion1-31_8-al-20_9/eGraduados_Inicio_Iteracion1_PlanificacionTemporal.xlsx
+++ b/A-Documentacion/A-Inicio/Iteracion1-31_8-al-20_9/eGraduados_Inicio_Iteracion1_PlanificacionTemporal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\eGraduados\A-Documentacion\A-Inicio\Iteracion1-31_8-al-20_9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2293724D-AE2C-4654-99A5-8BEDFDF513CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DC5D76-582E-4B66-AD6B-772A0362323A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{C157A7F2-5B1B-4E06-B43B-1F6A14E9BE8B}"/>
   </bookViews>
@@ -725,7 +725,7 @@
       <c r="I11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="7"/>
+      <c r="J11" s="6"/>
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C12" s="1">
@@ -789,7 +789,7 @@
       <c r="I14" s="1">
         <v>6</v>
       </c>
-      <c r="J14" s="7"/>
+      <c r="J14" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>